<commit_message>
W01 D1 checkpoint: family rebuilds in progress (decks, notebooks, exercises, companion, reading), not yet verified
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUygQmVJCQfNFYFAEwJdgB
</commit_message>
<xml_diff>
--- a/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
+++ b/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tree" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discount" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Typical" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lifts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,8 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,21 +39,33 @@
       <sz val="16"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <color rgb="001A1440"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="006B6690"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001A0F5C"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001A0F5C"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -62,12 +77,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A0F5C"/>
+        <fgColor rgb="00FFF4C2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF4C2"/>
+        <fgColor rgb="001A0F5C"/>
       </patternFill>
     </fill>
     <fill>
@@ -76,7 +91,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -98,24 +113,77 @@
         <color rgb="00CFC9EE"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CFC9EE"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CFC9EE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CFC9EE"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CFC9EE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CFC9EE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CFC9EE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CFC9EE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CFC9EE"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -481,58 +549,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The question before the budget: the decision tool</t>
+          <t>Is acquisition the short branch? The decision tool</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kalpa Retail, Week 1, Monday. Four decisions the day taught, one tab each, and an Export tab that assembles the brief.</t>
+          <t>Kalpa Retail, Week 1, Monday. Meera Raghavan, CEO, asked what sales is made of and whether acquisition is even the branch that is short, before she signs marketing's Rs 12 crore.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Yellow cells are inputs; every other number and sentence is a live formula.</t>
+          <t>The workbook holds the five decisions the day taught, one tab each, and an Export tab that assembles the brief to Meera.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Each tab carries one planted defect in one formula. Read the tab's check line first, find the cell, fix it, and watch the verdict change.</t>
+          <t>Yellow cells are inputs you may change; every other number and sentence is a live formula.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>The Export tab releases the paste-ready brief only when all four tabs pass their checks, so fixing one tab does not clear it.</t>
+          <t>Each tab carries one planted defect in one formula: the day's trap, written as a spreadsheet mistake. Read the tab's check line first, find the cell, fix the formula, and watch the verdict change.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Sales: which total is sales. Tree: do the branch moves reach the plan. Average: mean or median. Discount: does the discount pay.</t>
+          <t>The Export tab releases the brief only when all five tabs pass their checks, so fixing one tab does not clear it.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>The status totals on the Sales tab come from the day's thirty orders; every other number here is an input you can change.</t>
+          <t>Sales asks which total is sales. Customers asks whether customers are counted by rows or by id. Typical asks whether the typical order is the mean or the median. Lifts asks whether two lifts add or multiply. Channel asks what booked and delivered say about each channel on consumer orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>The figures on the tabs are aggregates of the day's 30 orders from 1 July to 26 September 2026, as the notebooks compute them. The few amounts marked invented are invented to show a mechanism and are not Kalpa records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>When you finish, use the tool on your own extract: replace the yellow cells, fix nothing, and read the verdicts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Yellow means input.</t>
         </is>
       </c>
     </row>
@@ -547,13 +636,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,201 +655,206 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Three honest readings of one word. The parts must add back to the whole before any total leaves the team.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Three honest readings of one word. A total leaves the team with its definition beside it.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Amount (Rs)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>delivered</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="8" t="n">
         <v>520790</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>returned</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="8" t="n">
         <v>14970</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>cancelled</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="8" t="n">
         <v>9050</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Reading</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Total (Rs)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>booked</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>all booked orders</t>
-        </is>
-      </c>
-      <c r="C10">
-        <f>C5+C6</f>
+      <c r="B10" s="6">
+        <f>B5+B6+B7</f>
+        <v/>
+      </c>
+      <c r="C10" s="9">
+        <f>C5+C6+C7</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>not cancelled</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>every order not cancelled</t>
-        </is>
-      </c>
-      <c r="C11">
-        <f>C5+C6</f>
+      <c r="B11" s="6">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C11" s="9">
+        <f>C5+C6+C7</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>delivered</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>delivered orders only</t>
-        </is>
-      </c>
-      <c r="C12">
+      <c r="B12" s="6">
+        <f>B5</f>
+        <v/>
+      </c>
+      <c r="C12" s="9">
         <f>C5</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Your reading</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>booked</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>The reading you give Meera</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>not cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <f>IF(C10=C5+C6+C7,"The parts add up to the booked total.","The parts do not add up to the booked total: one total leaves a row out. Fix it first.")</f>
+        <f>IF(C11=C10-C7,"The not-cancelled total is the booked total less the cancelled orders.","The not-cancelled total sits "&amp;IF(C11-(C10-C7)&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(C11-(C10-C7)),0)&gt;=100000,INT(ROUND(ABS(C11-(C10-C7)),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C11-(C10-C7)),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C11-(C10-C7)),0),1000),"000"),IF(ROUND(ABS(C11-(C10-C7)),0)&gt;=1000,INT(ROUND(ABS(C11-(C10-C7)),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(C11-(C10-C7)),0),1000),"000"),ROUND(ABS(C11-(C10-C7)),0)&amp;""))&amp;" above booked less cancelled: it still carries the cancelled orders, which never became sales. Fix it first.")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Chosen total</t>
-        </is>
-      </c>
-      <c r="B16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Chosen total (Rs)</t>
+        </is>
+      </c>
+      <c r="B16" s="9">
         <f>INDEX(C10:C12,MATCH(B14,A10:A12,0))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Its definition</t>
-        </is>
-      </c>
-      <c r="B17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Its orders</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
         <f>INDEX(B10:B12,MATCH(B14,A10:A12,0))</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B19" s="8">
-        <f>IF(C10&lt;&gt;C5+C6+C7,"Fix the total that leaves a row out before any number leaves the team.","Revenue, "&amp;B17&amp;", 1 July to 26 September: "&amp;"Rs "&amp;IF(ROUND(B16,0)&gt;=100000,INT(ROUND(B16,0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(B16,0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(B16,0),1000),"000"),IF(ROUND(B16,0)&gt;=1000,INT(ROUND(B16,0)/1000)&amp;","&amp;TEXT(MOD(ROUND(B16,0),1000),"000"),ROUND(B16,0)&amp;""))&amp;".")</f>
-        <v/>
-      </c>
+      <c r="B19" s="12">
+        <f>IF(C11&lt;&gt;C10-C7,"Fix the not-cancelled total before any number leaves the team.","Sales, "&amp;B14&amp;", 1 July to 26 September: "&amp;IF(B16&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B16),0)&gt;=100000,INT(ROUND(ABS(B16),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B16),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),IF(ROUND(ABS(B16),0)&gt;=1000,INT(ROUND(ABS(B16),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),ROUND(ABS(B16),0)&amp;""))&amp;" on "&amp;B17&amp;" orders"&amp;IF(B14="booked",", every order placed, cancelled and returned ones included.",", with "&amp;IF(C10-B16&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(C10-B16),0)&gt;=100000,INT(ROUND(ABS(C10-B16),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C10-B16),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C10-B16),0),1000),"000"),IF(ROUND(ABS(C10-B16),0)&gt;=1000,INT(ROUND(ABS(C10-B16),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(C10-B16),0),1000),"000"),ROUND(ABS(C10-B16),0)&amp;""))&amp;" and "&amp;(B10-B17)&amp;" orders of the booked total left out by the definition."))</f>
+        <v/>
+      </c>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="14" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
       </c>
-      <c r="B20">
-        <f>IF(C10=C5+C6+C7,1,0)</f>
+      <c r="B20" s="6">
+        <f>IF(C11=C10-C7,1,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B19:F19"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"booked,not cancelled,delivered"</formula1>
@@ -774,182 +870,193 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Do the branch moves reach the plan?</t>
+          <t>Customers by rows or by id?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Change each branch in percent. The tree multiplies its branches, and the extra discount comes off the top.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>A row is an order. How many customers placed each number of orders, and what that says about frequency.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Branch</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Change, percent</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Multiplier</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Orders placed in the window</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Orders they account for</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>customers</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C5">
-        <f>1+B5/100</f>
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C5" s="6">
+        <f>A5*B5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>orders per customer</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6">
-        <f>1+B6/100</f>
+      <c r="A6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="6">
+        <f>A6*B6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>items per order</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
+      <c r="A7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C7">
-        <f>1+B7/100</f>
+      <c r="C7" s="6">
+        <f>A7*B7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>price per item</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
+      <c r="A8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C8">
-        <f>1+B8/100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>extra discount, percent of gross</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <f>1-B9/100</f>
+      <c r="C8" s="6">
+        <f>A8*B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Orders (rows)</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
+        <f>SUMPRODUCT(A5:A8,B5:B8)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Revenue index, today at 100</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>100+B5+B6+B7+B8-B9</f>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>SUMPRODUCT(A5:A8,B5:B8)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>The product of the multipliers</t>
-        </is>
-      </c>
-      <c r="B12">
-        <f>100*C5*C6*C7*C8*C9</f>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Orders per customer</t>
+        </is>
+      </c>
+      <c r="B12" s="15">
+        <f>ROUND(B10/B11,2)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Customers who came back</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <f>SUM(B6:B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Customers who bought once</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
       </c>
-      <c r="B13" s="2">
-        <f>IF(ABS(B11-B12)&lt;0.05,"The index multiplies the branches, as the tree does.","The index and the product of the branches disagree: one formula adds what the tree multiplies. Fix it first.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>The plan</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="B15" s="2">
+        <f>IF(AND(B11=B10,B13&gt;0),"Customers equal orders, yet "&amp;B13&amp;" customers bought more than once: the customer cell is counting rows. Fix it first.","Customers count each id once, so repeat buyers show.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B16" s="8">
-        <f>IF(ABS(B11-B12)&gt;=0.05,"Fix the index that adds what the tree multiplies before reading any result.",IF(B11&gt;=B14,"The moves reach the plan: revenue index "&amp;TEXT(B11,"0.0")&amp;" against "&amp;B14&amp;".","The moves fall short: revenue index "&amp;TEXT(B11,"0.0")&amp;", "&amp;TEXT(B14-B11,"0.0")&amp;" points under the plan."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="B17" s="12">
+        <f>IF(AND(B11=B10,B13&gt;0),"Fix the customer count before you say anything about frequency.",IF(B13=0,"Every one of the "&amp;B11&amp;" customers bought once, so frequency has nothing to show yet and acquisition is the branch to test.",B11&amp;" customers placed "&amp;TEXT(B12,"0.00")&amp;" orders each; "&amp;B13&amp;" of them ("&amp;ROUND(100*B13/B11,0)&amp;" percent) came back and "&amp;B14&amp;" bought once, so frequency is a live branch before acquisition."))</f>
+        <v/>
+      </c>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="14" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
       </c>
-      <c r="B17">
-        <f>IF(ABS(B11-B12)&lt;0.05,1,0)</f>
+      <c r="B18" s="6">
+        <f>IF(B11=SUM(B5:B8),1,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B17:F17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -960,153 +1067,234 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Mean or median?</t>
+          <t>What does a typical order look like?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Five invented orders in the yellow cells, room for five more. The job the number does decides the average.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Kalpa's booked orders on the left; an invented list on the right shows why one order can move a mean.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Amounts (Rs)</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Kalpa, booked orders</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Booked revenue (Rs)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>544810</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Median order from notebook 3 (Rs)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Mean order (Rs)</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>ROUND(B5/B6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>The typical order you report (Rs)</t>
+        </is>
+      </c>
+      <c r="B9" s="9">
+        <f>B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Mean over median</t>
+        </is>
+      </c>
+      <c r="B10" s="16">
+        <f>ROUND(B8/B7,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>What is the number for?</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>a typical order</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>The check</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <f>IF(AND(B9=B8,B10&gt;=2),"The typical order reads the mean, which is "&amp;TEXT(B10,"0.0")&amp;" times the median: one large order is moving it. Fix it first.","The typical order reads the median, which one order cannot drag.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>IF(AND(B9=B8,B10&gt;=2),"Fix the typical order before it values anything.",IF(B11="a typical order","Report the median, "&amp;IF(B7&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B7),0)&gt;=100000,INT(ROUND(ABS(B7),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B7),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),IF(ROUND(ABS(B7),0)&gt;=1000,INT(ROUND(ABS(B7),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),ROUND(ABS(B7),0)&amp;""))&amp;", as the typical order: the mean of "&amp;IF(B8&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B8),0)&gt;=100000,INT(ROUND(ABS(B8),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B8),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),IF(ROUND(ABS(B8),0)&gt;=1000,INT(ROUND(ABS(B8),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),ROUND(ABS(B8),0)&amp;""))&amp;" is "&amp;TEXT(B10,"0.0")&amp;" times it, so a first order is worth about "&amp;IF(B7&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B7),0)&gt;=100000,INT(ROUND(ABS(B7),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B7),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),IF(ROUND(ABS(B7),0)&gt;=1000,INT(ROUND(ABS(B7),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),ROUND(ABS(B7),0)&amp;""))&amp;" to the acquisition case.","Use the mean, "&amp;IF(B8&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B8),0)&gt;=100000,INT(ROUND(ABS(B8),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B8),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),IF(ROUND(ABS(B8),0)&gt;=1000,INT(ROUND(ABS(B8),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),ROUND(ABS(B8),0)&amp;""))&amp;", on the tree, because it multiplies back to the total; say so beside it."))</f>
+        <v/>
+      </c>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Fixed, for the Export tab</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>IF(B9=B7,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Invented orders (Rs)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Invented list, measure</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
         <v>1900</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="D5">
-        <f>COUNT(A5:A14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="D18" s="9">
+        <f>ROUND(AVERAGE(A18:A22),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
         <v>2100</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Mean</t>
-        </is>
-      </c>
-      <c r="D6">
-        <f>AVERAGE(A5:A14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="D19" s="9">
+        <f>MEDIAN(A18:A22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
         <v>2200</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Median</t>
-        </is>
-      </c>
-      <c r="D7">
-        <f>AVERAGE(A5:A14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Orders above the mean</t>
+        </is>
+      </c>
+      <c r="D20" s="6">
+        <f>COUNTIF(A18:A22,"&gt;"&amp;D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
         <v>2400</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Mean over median</t>
-        </is>
-      </c>
-      <c r="D8">
-        <f>D6/D7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
         <v>90000</v>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>The check</t>
-        </is>
-      </c>
-      <c r="D9" s="2">
-        <f>IF(AND(D7=D6,MAX(A5:A14)&gt;5*MIN(A5:A14)),"The median equals the mean on a list whose largest value is many times its smallest: check the median formula. Fix it first.","The median is the middle of the sorted list.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>What is the number for?</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>a typical order</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="D13" s="8">
-        <f>IF(AND(D7=D6,MAX(A5:A14)&gt;5*MIN(A5:A14)),"Fix the median formula before choosing an average.",IF(D11="a typical order","Report the median, "&amp;"Rs "&amp;IF(ROUND(D7,0)&gt;=100000,INT(ROUND(D7,0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(D7,0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(D7,0),1000),"000"),IF(ROUND(D7,0)&gt;=1000,INT(ROUND(D7,0)/1000)&amp;","&amp;TEXT(MOD(ROUND(D7,0),1000),"000"),ROUND(D7,0)&amp;""))&amp;", as the typical order, and name the largest order on its own line.",IF(D11="a total that must add up","Use the mean, "&amp;"Rs "&amp;IF(ROUND(D6,0)&gt;=100000,INT(ROUND(D6,0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(D6,0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(D6,0),1000),"000"),IF(ROUND(D6,0)&gt;=1000,INT(ROUND(D6,0)/1000)&amp;","&amp;TEXT(MOD(ROUND(D6,0),1000),"000"),ROUND(D6,0)&amp;""))&amp;", because it multiplies back to the total.","Report both: the mean "&amp;"Rs "&amp;IF(ROUND(D6,0)&gt;=100000,INT(ROUND(D6,0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(D6,0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(D6,0),1000),"000"),IF(ROUND(D6,0)&gt;=1000,INT(ROUND(D6,0)/1000)&amp;","&amp;TEXT(MOD(ROUND(D6,0),1000),"000"),ROUND(D6,0)&amp;""))&amp;" and the median "&amp;"Rs "&amp;IF(ROUND(D7,0)&gt;=100000,INT(ROUND(D7,0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(D7,0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(D7,0),1000),"000"),IF(ROUND(D7,0)&gt;=1000,INT(ROUND(D7,0)/1000)&amp;","&amp;TEXT(MOD(ROUND(D7,0),1000),"000"),ROUND(D7,0)&amp;""))&amp;"; a gap of "&amp;TEXT(D8,"0.0")&amp;" times is itself a finding.")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n"/>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Fixed, for the Export tab</t>
-        </is>
-      </c>
-      <c r="D14">
-        <f>IF(D7=MEDIAN(A5:A14),1,0)</f>
-        <v/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>These five amounts are invented; change the last one to see the mean move and the median stay.</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B14:F14"/>
+  </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"a typical order,a total that must add up,a first look at a file"</formula1>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"a typical order,a total that must add up"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1119,117 +1307,203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Does the discount pay?</t>
+          <t>Do two lifts add or multiply?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>A discount trades margin for quantity. It pays only when volume rises by more than the price falls.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Revenue is customers times orders per customer times average order value, so lifts on its branches multiply.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Revenue today (Rs)</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>544810</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Discount, percent off</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Change, percent</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Multiplier</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>customers</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="6">
+        <f>1+B6/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>orders per customer</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="6">
+        <f>1+B7/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>average order value</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="6">
+        <f>1+B8/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>The growth plan, percent</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Expected volume lift, percent</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Revenue multiple against today</t>
-        </is>
-      </c>
-      <c r="B8">
-        <f>(1+B6/100)*(1-B5/100)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Break-even volume lift, percent</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>B5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Revenue if the lifts were added (Rs)</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>ROUND(B4*(1+(B6+B7+B8)/100),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>New revenue (Rs)</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>ROUND(B4*(1+(B6+B7+B8)/100),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Through the tree (Rs)</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>ROUND(B4*C6*C7*C8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Growth, percent</t>
+        </is>
+      </c>
+      <c r="B15" s="16">
+        <f>ROUND(100*(B13/B4-1),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
       </c>
-      <c r="B10" s="2">
-        <f>IF(ABS((1+B9/100)*(1-B5/100)-1)&lt;0.0005,"At the break-even lift the discount leaves revenue where it was.","At the stated break-even lift revenue still falls: the break-even formula is wrong. Fix it first.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="B16" s="2">
+        <f>IF(ABS(B13-B14)&gt;1,"New revenue and the product of the branches disagree by "&amp;IF(B14-B13&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B14-B13),0)&gt;=100000,INT(ROUND(ABS(B14-B13),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B14-B13),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B14-B13),0),1000),"000"),IF(ROUND(ABS(B14-B13),0)&gt;=1000,INT(ROUND(ABS(B14-B13),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B14-B13),0),1000),"000"),ROUND(ABS(B14-B13),0)&amp;""))&amp;": the new revenue adds what the tree multiplies. Fix it first.","New revenue multiplies the branches, as the tree does.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B12" s="8">
-        <f>IF(ABS((1+B9/100)*(1-B5/100)-1)&gt;=0.0005,"Fix the break-even formula before judging the discount.",IF(B8&gt;=1,"The discount pays: revenue ends at "&amp;TEXT(B8,"0.000")&amp;" of today.","The discount loses: revenue ends at "&amp;TEXT(B8,"0.000")&amp;" of today, and it needs "&amp;TEXT(B9,"0.0")&amp;" percent more volume just to stand still."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="B18" s="12">
+        <f>IF(ABS(B13-B14)&gt;1,"Fix the new revenue before you quote any growth.","Through the tree, revenue moves from "&amp;IF(B4&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B4),0)&gt;=100000,INT(ROUND(ABS(B4),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B4),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B4),0),1000),"000"),IF(ROUND(ABS(B4),0)&gt;=1000,INT(ROUND(ABS(B4),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B4),0),1000),"000"),ROUND(ABS(B4),0)&amp;""))&amp;" to "&amp;IF(B13&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B13),0)&gt;=100000,INT(ROUND(ABS(B13),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B13),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B13),0),1000),"000"),IF(ROUND(ABS(B13),0)&gt;=1000,INT(ROUND(ABS(B13),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B13),0),1000),"000"),ROUND(ABS(B13),0)&amp;""))&amp;", "&amp;IF(B15&gt;=0,"up ","down ")&amp;TEXT(ABS(B15),"0.0")&amp;" percent, which "&amp;IF(B15&gt;=B10,"reaches","misses")&amp;" the "&amp;B10&amp;" percent plan; adding the lifts would have said "&amp;IF(B12&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B12),0)&gt;=100000,INT(ROUND(ABS(B12),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B12),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B12),0),1000),"000"),IF(ROUND(ABS(B12),0)&gt;=1000,INT(ROUND(ABS(B12),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B12),0),1000),"000"),ROUND(ABS(B12),0)&amp;""))&amp;".")</f>
+        <v/>
+      </c>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="14" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Fixed, for the Export tab</t>
         </is>
       </c>
-      <c r="B13">
-        <f>IF(ABS((1+B9/100)*(1-B5/100)-1)&lt;0.0005,1,0)</f>
-        <v/>
+      <c r="B19" s="6">
+        <f>IF(ABS(B13-B14)&lt;=1,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Try the discount: set customers to 0, orders per customer to 10 for the extra quantity, and average order value to minus 15 for 15 percent off.</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B18:F18"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1240,59 +1514,324 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The brief, assembled</t>
+          <t>Booked against delivered, by channel</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Consumer orders only: the 29 orders outside the Business segment. Each channel split by what happened to its orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>The view you give Meera</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>The headline it replaces</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Store carried 91.6 percent of all booked revenue, Rs 4,98,920 of Rs 5,44,810, on every order in the file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Booked orders</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Booked (Rs)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Cancelled (Rs)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Returned (Rs)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Delivered (Rs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>18600</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9">
+        <f>C8-D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>27290</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>14970</v>
+      </c>
+      <c r="F9" s="9">
+        <f>C9-D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>store</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>18920</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>9050</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="9">
+        <f>C10-D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>All consumer orders</t>
+        </is>
+      </c>
+      <c r="B11" s="17">
+        <f>SUM(B8:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="17">
+        <f>SUM(C8:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="17">
+        <f>SUM(D8:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="17">
+        <f>SUM(E8:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="17">
+        <f>SUM(F8:F10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>The check</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <f>IF(F11+D11+E11&lt;&gt;C11,"Delivered, cancelled and returned add to "&amp;IF(F11+D11+E11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(F11+D11+E11),0)&gt;=100000,INT(ROUND(ABS(F11+D11+E11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(F11+D11+E11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(F11+D11+E11),0),1000),"000"),IF(ROUND(ABS(F11+D11+E11),0)&gt;=1000,INT(ROUND(ABS(F11+D11+E11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(F11+D11+E11),0),1000),"000"),ROUND(ABS(F11+D11+E11),0)&amp;""))&amp;" against "&amp;IF(C11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(C11),0)&gt;=100000,INT(ROUND(ABS(C11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C11),0),1000),"000"),IF(ROUND(ABS(C11),0)&gt;=1000,INT(ROUND(ABS(C11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(C11),0),1000),"000"),ROUND(ABS(C11),0)&amp;""))&amp;" booked: the delivered column still carries the returns. Fix it first.","Delivered, cancelled and returned add back to the booked total.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Leader in the chosen view</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>IF(B4="booked",INDEX(A8:A10,MATCH(MAX(C8:C10),C8:C10,0)),INDEX(A8:A10,MATCH(MAX(F8:F10),F8:F10,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Its amount (Rs)</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>IF(B4="booked",MAX(C8:C10),MAX(F8:F10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Of (Rs)</t>
+        </is>
+      </c>
+      <c r="B16" s="9">
+        <f>IF(B4="booked",C11,F11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B18" s="12">
+        <f>IF(F11+D11+E11&lt;&gt;C11,"Fix the delivered column before you rank any channel.","On consumer orders "&amp;B4&amp;", "&amp;B14&amp;" leads with "&amp;IF(B15&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B15),0)&gt;=100000,INT(ROUND(ABS(B15),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B15),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B15),0),1000),"000"),IF(ROUND(ABS(B15),0)&gt;=1000,INT(ROUND(ABS(B15),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B15),0),1000),"000"),ROUND(ABS(B15),0)&amp;""))&amp;" of "&amp;IF(B16&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B16),0)&gt;=100000,INT(ROUND(ABS(B16),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B16),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),IF(ROUND(ABS(B16),0)&gt;=1000,INT(ROUND(ABS(B16),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),ROUND(ABS(B16),0)&amp;""))&amp;"; returns took "&amp;IF(E11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(E11),0)&gt;=100000,INT(ROUND(ABS(E11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(E11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(E11),0),1000),"000"),IF(ROUND(ABS(E11),0)&gt;=1000,INT(ROUND(ABS(E11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(E11),0),1000),"000"),ROUND(ABS(E11),0)&amp;""))&amp;" and cancellations "&amp;IF(D11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(D11),0)&gt;=100000,INT(ROUND(ABS(D11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(D11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(D11),0),1000),"000"),IF(ROUND(ABS(D11),0)&gt;=1000,INT(ROUND(ABS(D11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(D11),0),1000),"000"),ROUND(ABS(D11),0)&amp;""))&amp;", so the channel view adds two leaks to name and leaves frequency first standing.")</f>
+        <v/>
+      </c>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="14" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Fixed, for the Export tab</t>
+        </is>
+      </c>
+      <c r="B19" s="6">
+        <f>IF(F11+D11+E11=C11,1,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B13:F13"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"booked,delivered"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The brief to Meera, assembled</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Released only when every tab's check passes. Paste the brief into the note to Meera.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Tabs fixed</t>
         </is>
       </c>
-      <c r="B4">
-        <f>Sales!B20+Tree!B17+Average!D14+Discount!B13</f>
+      <c r="B4" s="6">
+        <f>Sales!B20+Customers!B18+Typical!B15+Lifts!B19+Channel!B19</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="B5" s="8">
-        <f>IF(B4=4,"Ready to paste into the note to Meera.","Not ready: "&amp;(4-B4)&amp;" of the four tabs still carry a defect to fix first.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="B5" s="12">
+        <f>IF(B4=5,"Ready to paste into the note to Meera.","Not ready: tabs still carrying a defect, "&amp;(5-B4)&amp;" of five.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="170" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Paste-ready brief</t>
         </is>
       </c>
       <c r="B7" s="2">
-        <f>IF(B4=4,"Sales: "&amp;Sales!B19&amp;CHAR(10)&amp;"Tree: "&amp;Tree!B16&amp;CHAR(10)&amp;"Average: "&amp;Average!D13&amp;CHAR(10)&amp;"Discount: "&amp;Discount!B12,"The brief assembles once every tab passes its check.")</f>
+        <f>IF(B4=5,Sales!B19&amp;CHAR(10)&amp;"Customers: "&amp;Customers!B17&amp;CHAR(10)&amp;"Typical order: "&amp;Typical!B14&amp;CHAR(10)&amp;"Lifts: "&amp;Lifts!B18&amp;CHAR(10)&amp;"Channels: "&amp;Channel!B18&amp;CHAR(10)&amp;"Recommendation: open frequency before acquisition; one window cannot show which branch moved, so hold the Rs 12 crore until Tuesday's two quarters.","The brief assembles once every tab passes its check.")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
W01 D1 checkpoint: files in progress, not yet verified
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUygQmVJCQfNFYFAEwJdgB
</commit_message>
<xml_diff>
--- a/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
+++ b/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
@@ -1067,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="D18" s="9">
-        <f>ROUND(AVERAGE(A18:A22),0)</f>
+        <f>ROUND(AVERAGE(A18:A23),0)</f>
         <v/>
       </c>
     </row>
@@ -1252,13 +1252,13 @@
         </is>
       </c>
       <c r="D19" s="9">
-        <f>MEDIAN(A18:A22)</f>
+        <f>MEDIAN(A18:A23)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>2200</v>
+        <v>2300</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
@@ -1266,7 +1266,7 @@
         </is>
       </c>
       <c r="D20" s="6">
-        <f>COUNTIF(A18:A22,"&gt;"&amp;D18)</f>
+        <f>COUNTIF(A18:A23,"&gt;"&amp;D18)</f>
         <v/>
       </c>
     </row>
@@ -1277,13 +1277,18 @@
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
         <v>90000</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>These five amounts are invented; change the last one to see the mean move and the median stay.</t>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>These six amounts are invented; clear the last one to see the mean fall back while the median barely moves.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
W01 D1 reading and trainer: day sheet on the domain-first grid, notes per chapter, board work with the story's drawings, six-crux cheat sheet, Kahoot by chapter, companion walk and two new workbook tabs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UyiPuGXFQ9xh3hKJPZUz8p
</commit_message>
<xml_diff>
--- a/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
+++ b/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Typical" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lifts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fraction" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Typical" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lifts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edge" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +574,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>The workbook holds the five decisions the day taught, one tab each, and an Export tab that assembles the brief to Meera.</t>
+          <t>The workbook holds the seven decisions the day taught, one tab each, and an Export tab that assembles the brief to Meera.</t>
         </is>
       </c>
     </row>
@@ -593,14 +595,14 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>The Export tab releases the brief only when all five tabs pass their checks, so fixing one tab does not clear it.</t>
+          <t>The Export tab releases the brief only when all seven tabs pass their checks, so fixing one tab does not clear it.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sales asks which total is sales. Customers asks whether customers are counted by rows or by id. Typical asks whether the typical order is the mean or the median. Lifts asks whether two lifts add or multiply. Channel asks what booked and delivered say about each channel on consumer orders.</t>
+          <t>Sales asks which total is sales. Fraction asks whether the AOV is one definition over the same definition. Customers asks whether customers are counted by rows or by id. Typical asks whether the typical order is the mean or the median. Lifts asks whether two lifts add or multiply. Edge asks whether a one-time buyer is lost or too recent to judge. Channel asks what booked and delivered say about each channel on consumer orders.</t>
         </is>
       </c>
     </row>
@@ -870,6 +872,187 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Is the AOV one definition over the same definition?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>A branch is a fraction on one definition. Orders times AOV has to land on that definition's revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Revenue (Rs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>booked</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>544810</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>520790</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>The definition you report</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Its orders</t>
+        </is>
+      </c>
+      <c r="B9" s="6">
+        <f>INDEX(B5:B6,MATCH(B8,A5:A6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Its revenue (Rs)</t>
+        </is>
+      </c>
+      <c r="B10" s="9">
+        <f>INDEX(C5:C6,MATCH(B8,A5:A6,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>AOV (Rs)</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>ROUND(C5/B9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Orders x AOV (Rs)</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>B9*B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>The check</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <f>IF(ABS(B12-B10)&lt;=B9,"Orders times AOV lands on "&amp;B8&amp;" revenue.","Orders times AOV comes to "&amp;IF(B12&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B12),0)&gt;=100000,INT(ROUND(ABS(B12),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B12),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B12),0),1000),"000"),IF(ROUND(ABS(B12),0)&gt;=1000,INT(ROUND(ABS(B12),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B12),0),1000),"000"),ROUND(ABS(B12),0)&amp;""))&amp;", which lands on no revenue: the AOV divides one definition's rupees by another's orders. Fix it first.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>IF(ABS(B12-B10)&gt;B9,"Fix the AOV before it values any order.","AOV on the "&amp;B8&amp;" definition is "&amp;IF(B11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B11),0)&gt;=100000,INT(ROUND(ABS(B11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B11),0),1000),"000"),IF(ROUND(ABS(B11),0)&gt;=1000,INT(ROUND(ABS(B11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B11),0),1000),"000"),ROUND(ABS(B11),0)&amp;""))&amp;" on "&amp;B9&amp;" orders, and it multiplies back to "&amp;IF(B10&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B10),0)&gt;=100000,INT(ROUND(ABS(B10),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B10),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B10),0),1000),"000"),IF(ROUND(ABS(B10),0)&gt;=1000,INT(ROUND(ABS(B10),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B10),0),1000),"000"),ROUND(ABS(B10),0)&amp;""))&amp;".")</f>
+        <v/>
+      </c>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="14" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Fixed, for the Export tab</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>IF(B11=ROUND(B10/B9,0),1,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B13:F13"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"booked,delivered"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1061,7 +1244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1306,7 +1489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1513,7 +1696,168 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lost, or too recent to judge?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>A one-time buyer is not lost until they have had the usual time to come back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Came back</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Bought once</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Median days between a first and second order</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>One-time buyers who bought inside the last gap</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Had time and did not come back</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Share of customers who look lost, percent</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
+        <f>ROUND(100*B11/B5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>The check</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <f>IF(AND(B11=B7,B9&gt;0),"The count treats all "&amp;B7&amp;" one-time buyers as lost, although "&amp;B9&amp;" bought inside the last "&amp;B8&amp;" days. Fix it first.","The count holds back the "&amp;B9&amp;" one-time buyers who have not had "&amp;B8&amp;" days.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>IF(AND(B11=B7,B9&gt;0),"Fix the lost count before the sentence calls anyone lost.",B6&amp;" came back, "&amp;B11&amp;" had time and did not, and "&amp;B9&amp;" bought too recently to judge, so at most "&amp;B12&amp;" percent of customers look lost.")</f>
+        <v/>
+      </c>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="14" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Fixed, for the Export tab</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>IF(B11=B7-B9,1,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B13:F13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1780,7 +2124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1814,7 +2158,7 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>Sales!B20+Customers!B18+Typical!B15+Lifts!B19+Channel!B19</f>
+        <f>Sales!B20+Fraction!B16+Customers!B18+Typical!B15+Lifts!B19+Edge!B16+Channel!B19</f>
         <v/>
       </c>
     </row>
@@ -1825,7 +2169,7 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>IF(B4=5,"Ready to paste into the note to Meera.","Not ready: tabs still carrying a defect, "&amp;(5-B4)&amp;" of five.")</f>
+        <f>IF(B4=7,"Ready to paste into the note to Meera.","Not ready: tabs still carrying a defect, "&amp;(7-B4)&amp;" of seven.")</f>
         <v/>
       </c>
     </row>
@@ -1836,7 +2180,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>IF(B4=5,Sales!B19&amp;CHAR(10)&amp;"Customers: "&amp;Customers!B17&amp;CHAR(10)&amp;"Typical order: "&amp;Typical!B14&amp;CHAR(10)&amp;"Lifts: "&amp;Lifts!B18&amp;CHAR(10)&amp;"Channels: "&amp;Channel!B18&amp;CHAR(10)&amp;"Recommendation: open frequency before acquisition; one window cannot show which branch moved, so hold the Rs 12 crore until Tuesday's two quarters.","The brief assembles once every tab passes its check.")</f>
+        <f>IF(B4=7,Sales!B19&amp;CHAR(10)&amp;"Order value: "&amp;Fraction!B15&amp;CHAR(10)&amp;"Customers: "&amp;Customers!B17&amp;CHAR(10)&amp;"Typical order: "&amp;Typical!B14&amp;CHAR(10)&amp;"Lifts: "&amp;Lifts!B18&amp;CHAR(10)&amp;"The window: "&amp;Edge!B15&amp;CHAR(10)&amp;"Channels: "&amp;Channel!B18&amp;CHAR(10)&amp;"Recommendation: open frequency before acquisition; one window cannot show which branch moved, so hold the Rs 12 crore until Tuesday's two quarters.","The brief assembles once every tab passes its check.")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
W01 D1 depth loop second runs: identity shown on its own denominator, 14-month payback asserted, cued items neutralised, the repeat-order leak stated as counted, two slides folded into notes, seven sections on the afternoon cover, not-cancelled items, slogans rewritten, anchor as one row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UyiPuGXFQ9xh3hKJPZUz8p
</commit_message>
<xml_diff>
--- a/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
+++ b/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
@@ -1523,11 +1523,11 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Revenue today (Rs)</t>
+          <t>Everyday revenue today, the 29 orders the plan is sized on (Rs)</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>544810</v>
+        <v>64810</v>
       </c>
     </row>
     <row r="5">
@@ -1792,7 +1792,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Had time and did not come back</t>
+          <t>Past the usual gap, no second order</t>
         </is>
       </c>
       <c r="B11" s="6">
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B15" s="12">
-        <f>IF(AND(B11=B7,B9&gt;0),"Fix the lost count before the sentence calls anyone lost.",B6&amp;" came back, "&amp;B11&amp;" had time and did not, and "&amp;B9&amp;" bought too recently to judge, so at most "&amp;B12&amp;" percent of customers look lost.")</f>
+        <f>IF(AND(B11=B7,B9&gt;0),"Fix the lost count before the sentence calls anyone lost.",B6&amp;" came back, "&amp;B11&amp;" are past the usual gap, and "&amp;B9&amp;" bought too recently to judge, so at most "&amp;B12&amp;" percent of customers look lost.")</f>
         <v/>
       </c>
       <c r="C15" s="13" t="n"/>

</xml_diff>

<commit_message>
W01 D1 v3 recheck, checkpoint: question ladder, plant ruling and deck depth passes in progress, not yet verified
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MopBs5gTZd6CHnuNPtPfdF
</commit_message>
<xml_diff>
--- a/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
+++ b/content/W01/D1/demos/C2_W01_D01_decision_tool_STUDENT.xlsx
@@ -163,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -185,6 +185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -560,14 +561,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Is acquisition the short branch? The decision tool</t>
+          <t>Is acquisition even the branch that is short?</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kalpa Retail, Week 1, Monday. Meera Raghavan, CEO, asked what sales is made of and whether acquisition is even the branch that is short, before she signs marketing's Rs 12 crore.</t>
+          <t>This is the decision tool for Kalpa Retail, Week 1, Monday. Meera Raghavan, CEO, asked what sales is made of and whether acquisition is even the branch that is short, before she signs marketing's Rs 12 crore.</t>
         </is>
       </c>
     </row>
@@ -602,7 +603,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sales asks which total is sales. Fraction asks whether the AOV is one definition over the same definition. Customers asks whether customers are counted by rows or by id. Typical asks whether the typical order is the mean or the median. Lifts asks whether two lifts add or multiply. Edge asks whether a one-time buyer is lost or too recent to judge. Channel asks what booked and delivered say about each channel on consumer orders.</t>
+          <t>Each tab's title is the question it answers. Sales asks which total is sales, Fraction whether the AOV is one definition over the same definition, Customers whether customers are counted by rows or by id, and Typical whether the typical order is the mean or the median. Lifts asks whether two lifts add or multiply, Edge whether a one-time buyer is lost or too recent to judge, and Channel what each channel books and keeps in the three consumer segments Meera's plan concerns, Retail-Core, Retail-Plus and Student.</t>
         </is>
       </c>
     </row>
@@ -652,14 +653,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Which total is sales?</t>
+          <t>Which of the file's totals should Meera call sales?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Three honest readings of one word. A total leaves the team with its definition beside it.</t>
+          <t>One word has three honest readings, so a total leaves the team with its definition beside it.</t>
         </is>
       </c>
     </row>
@@ -784,7 +785,7 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>The reading you give Meera</t>
+          <t>Which reading do you give Meera?</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -886,7 +887,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Is the AOV one definition over the same definition?</t>
+          <t>Is the average order value one definition over the same definition?</t>
         </is>
       </c>
     </row>
@@ -943,7 +944,7 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>The definition you report</t>
+          <t>Which definition do you report?</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1067,14 +1068,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Customers by rows or by id?</t>
+          <t>Are Kalpa's customers counted by rows or by id?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>A row is an order. How many customers placed each number of orders, and what that says about frequency.</t>
+          <t>A row is an order, so the table counts customers by how many orders each placed, which is what the frequency branch is made of.</t>
         </is>
       </c>
     </row>
@@ -1264,14 +1265,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>What does a typical order look like?</t>
+          <t>What does a typical Kalpa order look like, so that one large order cannot move it?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Kalpa's booked orders on the left; an invented list on the right shows why one order can move a mean.</t>
+          <t>Kalpa's booked orders sit at the top, and the invented list below them shows how one order can move a mean.</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1311,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Median order from notebook 3 (Rs)</t>
+          <t>Median order from notebook 04 (Rs)</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
@@ -1369,7 +1370,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>IF(AND(B9=B8,B10&gt;=2),"The typical order reads the mean, which is "&amp;TEXT(B10,"0.0")&amp;" times the median: one large order is moving it. Fix it first.","The typical order reads the median, which one order cannot drag.")</f>
+        <f>IF(AND(B9=B8,B10&gt;=2),"The typical order reads the mean, which is "&amp;TEXT(B10,"0.0")&amp;" times the median, so the largest orders are dragging it. Fix it first.","The typical order reads the median, which one order cannot drag.")</f>
         <v/>
       </c>
     </row>
@@ -1380,7 +1381,7 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>IF(AND(B9=B8,B10&gt;=2),"Fix the typical order before it values anything.",IF(B11="a typical order","Report the median, "&amp;IF(B7&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B7),0)&gt;=100000,INT(ROUND(ABS(B7),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B7),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),IF(ROUND(ABS(B7),0)&gt;=1000,INT(ROUND(ABS(B7),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),ROUND(ABS(B7),0)&amp;""))&amp;", as the typical order: the mean of "&amp;IF(B8&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B8),0)&gt;=100000,INT(ROUND(ABS(B8),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B8),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),IF(ROUND(ABS(B8),0)&gt;=1000,INT(ROUND(ABS(B8),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),ROUND(ABS(B8),0)&amp;""))&amp;" is "&amp;TEXT(B10,"0.0")&amp;" times it, so a first order is worth about "&amp;IF(B7&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B7),0)&gt;=100000,INT(ROUND(ABS(B7),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B7),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),IF(ROUND(ABS(B7),0)&gt;=1000,INT(ROUND(ABS(B7),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),ROUND(ABS(B7),0)&amp;""))&amp;" to the acquisition case.","Use the mean, "&amp;IF(B8&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B8),0)&gt;=100000,INT(ROUND(ABS(B8),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B8),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),IF(ROUND(ABS(B8),0)&gt;=1000,INT(ROUND(ABS(B8),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),ROUND(ABS(B8),0)&amp;""))&amp;", on the tree, because it multiplies back to the total; say so beside it."))</f>
+        <f>IF(AND(B9=B8,B10&gt;=2),"Fix the typical order before it values anything.",IF(B11="a typical order","Report the median, "&amp;IF(B7&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B7),0)&gt;=100000,INT(ROUND(ABS(B7),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B7),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),IF(ROUND(ABS(B7),0)&gt;=1000,INT(ROUND(ABS(B7),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B7),0),1000),"000"),ROUND(ABS(B7),0)&amp;""))&amp;", as the typical order: the mean of "&amp;IF(B8&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B8),0)&gt;=100000,INT(ROUND(ABS(B8),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B8),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),IF(ROUND(ABS(B8),0)&gt;=1000,INT(ROUND(ABS(B8),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),ROUND(ABS(B8),0)&amp;""))&amp;" is "&amp;TEXT(B10,"0.0")&amp;" times it, so the mean describes no typical first order.","Use the mean, "&amp;IF(B8&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B8),0)&gt;=100000,INT(ROUND(ABS(B8),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B8),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),IF(ROUND(ABS(B8),0)&gt;=1000,INT(ROUND(ABS(B8),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B8),0),1000),"000"),ROUND(ABS(B8),0)&amp;""))&amp;", on the tree, because it multiplies back to the total; say so beside it."))</f>
         <v/>
       </c>
       <c r="C14" s="13" t="n"/>
@@ -1509,7 +1510,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Do two lifts add or multiply?</t>
+          <t>Do two 10 percent lifts on the tree add up, or multiply?</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1524,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Everyday revenue today, the 29 orders the plan is sized on (Rs)</t>
+          <t>Consumer revenue today, in the three consumer segments the plan is sized on (Rs)</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
@@ -1592,7 +1593,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>The growth plan, percent</t>
+          <t>How much growth does the plan ask for, in percent?</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
@@ -1716,14 +1717,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lost, or too recent to judge?</t>
+          <t>Is a one-time buyer lost, or too recent to judge?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>A one-time buyer is not lost until they have had the usual time to come back.</t>
+          <t>A one-time buyer counts as lost only after they have had the usual time to come back.</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1868,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -1877,21 +1878,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Booked against delivered, by channel</t>
+          <t>What does each channel book and keep in the three consumer segments?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Consumer orders only: the 29 orders outside the Business segment. Each channel split by what happened to its orders.</t>
+          <t>The consumer view keeps the orders whose segment is Retail-Core, Retail-Plus or Student, the three consumer segments Meera's plan concerns, and each channel is split by what happened to its orders.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>The view you give Meera</t>
+          <t>Which view do you give Meera?</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1920,7 +1921,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Booked orders</t>
+          <t>Share of booked, percent</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1950,8 +1951,9 @@
           <t>app</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>10</v>
+      <c r="B8" s="16">
+        <f>ROUND(100*C8/C$11,1)</f>
+        <v/>
       </c>
       <c r="C8" s="8" t="n">
         <v>18600</v>
@@ -1973,8 +1975,9 @@
           <t>web</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>10</v>
+      <c r="B9" s="16">
+        <f>ROUND(100*C9/C$11,1)</f>
+        <v/>
       </c>
       <c r="C9" s="8" t="n">
         <v>27290</v>
@@ -1996,8 +1999,9 @@
           <t>store</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
-        <v>9</v>
+      <c r="B10" s="16">
+        <f>ROUND(100*C10/C$11,1)</f>
+        <v/>
       </c>
       <c r="C10" s="8" t="n">
         <v>18920</v>
@@ -2016,26 +2020,26 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>All consumer orders</t>
+          <t>The consumer view</t>
         </is>
       </c>
       <c r="B11" s="17">
         <f>SUM(B8:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="18">
         <f>SUM(C8:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="18">
         <f>SUM(D8:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="18">
         <f>SUM(E8:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="18">
         <f>SUM(F8:F10)</f>
         <v/>
       </c>
@@ -2091,7 +2095,7 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>IF(F11+D11+E11&lt;&gt;C11,"Fix the delivered column before you rank any channel.","On consumer orders "&amp;B4&amp;", "&amp;B14&amp;" leads with "&amp;IF(B15&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B15),0)&gt;=100000,INT(ROUND(ABS(B15),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B15),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B15),0),1000),"000"),IF(ROUND(ABS(B15),0)&gt;=1000,INT(ROUND(ABS(B15),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B15),0),1000),"000"),ROUND(ABS(B15),0)&amp;""))&amp;" of "&amp;IF(B16&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B16),0)&gt;=100000,INT(ROUND(ABS(B16),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B16),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),IF(ROUND(ABS(B16),0)&gt;=1000,INT(ROUND(ABS(B16),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),ROUND(ABS(B16),0)&amp;""))&amp;"; returns took "&amp;IF(E11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(E11),0)&gt;=100000,INT(ROUND(ABS(E11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(E11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(E11),0),1000),"000"),IF(ROUND(ABS(E11),0)&gt;=1000,INT(ROUND(ABS(E11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(E11),0),1000),"000"),ROUND(ABS(E11),0)&amp;""))&amp;" and cancellations "&amp;IF(D11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(D11),0)&gt;=100000,INT(ROUND(ABS(D11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(D11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(D11),0),1000),"000"),IF(ROUND(ABS(D11),0)&gt;=1000,INT(ROUND(ABS(D11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(D11),0),1000),"000"),ROUND(ABS(D11),0)&amp;""))&amp;", so the channel view adds two leaks to name and leaves frequency first standing.")</f>
+        <f>IF(F11+D11+E11&lt;&gt;C11,"Fix the delivered column before you rank any channel.","In the consumer view, "&amp;B4&amp;", "&amp;B14&amp;" leads with "&amp;IF(B15&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B15),0)&gt;=100000,INT(ROUND(ABS(B15),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B15),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B15),0),1000),"000"),IF(ROUND(ABS(B15),0)&gt;=1000,INT(ROUND(ABS(B15),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B15),0),1000),"000"),ROUND(ABS(B15),0)&amp;""))&amp;" of "&amp;IF(B16&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(B16),0)&gt;=100000,INT(ROUND(ABS(B16),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B16),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),IF(ROUND(ABS(B16),0)&gt;=1000,INT(ROUND(ABS(B16),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B16),0),1000),"000"),ROUND(ABS(B16),0)&amp;""))&amp;"; returns took "&amp;IF(E11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(E11),0)&gt;=100000,INT(ROUND(ABS(E11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(E11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(E11),0),1000),"000"),IF(ROUND(ABS(E11),0)&gt;=1000,INT(ROUND(ABS(E11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(E11),0),1000),"000"),ROUND(ABS(E11),0)&amp;""))&amp;" and cancellations "&amp;IF(D11&lt;0,"minus ","")&amp;"Rs "&amp;IF(ROUND(ABS(D11),0)&gt;=100000,INT(ROUND(ABS(D11),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(D11),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(D11),0),1000),"000"),IF(ROUND(ABS(D11),0)&gt;=1000,INT(ROUND(ABS(D11),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(D11),0),1000),"000"),ROUND(ABS(D11),0)&amp;""))&amp;", so the channel view adds two leaks to name and leaves frequency first standing.")</f>
         <v/>
       </c>
       <c r="C18" s="13" t="n"/>
@@ -2140,14 +2144,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The brief to Meera, assembled</t>
+          <t>Is the brief to Meera ready to paste?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Released only when every tab's check passes. Paste the brief into the note to Meera.</t>
+          <t>The brief is released only when every tab's check passes; then paste it into the note to Meera.</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2173,7 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>IF(B4=7,"Ready to paste into the note to Meera.","Not ready: tabs still carrying a defect, "&amp;(7-B4)&amp;" of seven.")</f>
+        <f>IF(B4=7,"Ready to paste into the note to Meera.","Not ready: "&amp;IF(B4=6,"1 of 7 tabs still carries a defect.",(7-B4)&amp;" of 7 tabs still carry a defect."))</f>
         <v/>
       </c>
     </row>

</xml_diff>